<commit_message>
Unificar centros Arica - solo Oficina Ventas Arica
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -1149,7 +1149,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -5241,7 +5241,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -7112,7 +7112,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -8318,7 +8318,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -8353,7 +8353,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -8388,7 +8388,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -8423,7 +8423,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -8493,7 +8493,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -8563,7 +8563,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -8598,7 +8598,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -8633,7 +8633,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -8668,7 +8668,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -8703,7 +8703,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -8738,7 +8738,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -10679,7 +10679,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -10714,7 +10714,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -10749,7 +10749,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -10784,7 +10784,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -10819,7 +10819,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -10854,7 +10854,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -10889,7 +10889,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -10959,7 +10959,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -13250,7 +13250,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -13285,7 +13285,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -23556,7 +23556,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
@@ -23591,7 +23591,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -23626,7 +23626,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -23661,7 +23661,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
@@ -23696,7 +23696,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Oficina de Ventas Arica</t>
+          <t>Oficina Ventas Arica</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">

</xml_diff>

<commit_message>
fix: agregar precio Copiapó faltante para código 1000810 (TC2- ANEXOF)
Mismo caso que el código 1000180: TC2- ANEXOF solo tenía precio para
Arica/Antofagasta/Iquique, no para Copiapó. Se agrega la fila de
Copiapó copiando el valor de Arica ($65.000).

Confirmado con el usuario antes de aplicar (afecta el catálogo de
precios en producción).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -14023,7 +14023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G108"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="57.140625" customWidth="1" min="3" max="3"/>
@@ -17774,6 +17774,41 @@
       </c>
       <c r="G107" t="n">
         <v>150000</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>TC2- ANEXOF</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1000810</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G108" t="n">
+        <v>65000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: corregir 14 precios desalineados en base_datos.xlsx
9 ítems de Copiapó (SERVICIO CAÑERIAS, CONEXIONES, OBRAS CIVILES,
NORMALIZACIONES) y 4 de EQUIPO COMPRA DIRECTA (Arica/Iquique) tenían
precios muy por debajo (20-65%) del resto de los centros para el mismo
código. Se alinean al valor usado por los demás centros, igual que las
correcciones previas de Copiapó (7a01cb0, 20113ba).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -9176,7 +9176,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>7500</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="4">
@@ -9246,7 +9246,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>350</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="6">
@@ -9895,7 +9895,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>10000</v>
+        <v>37000</v>
       </c>
     </row>
     <row r="3">
@@ -9965,7 +9965,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>12784</v>
+        <v>27500</v>
       </c>
     </row>
     <row r="5">
@@ -10035,7 +10035,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>21840</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="7">
@@ -10070,7 +10070,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>21590</v>
+        <v>38500</v>
       </c>
     </row>
     <row r="8">
@@ -10140,7 +10140,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>9952</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="10">
@@ -12749,7 +12749,7 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>4800</v>
+        <v>11813</v>
       </c>
     </row>
     <row r="10">
@@ -15218,7 +15218,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>14000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="35">
@@ -18177,7 +18177,7 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>64330</v>
+        <v>134021</v>
       </c>
     </row>
     <row r="11">
@@ -18422,7 +18422,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>46</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18">
@@ -21047,7 +21047,7 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>45</v>
+        <v>67</v>
       </c>
     </row>
     <row r="93">
@@ -21397,7 +21397,7 @@
         </is>
       </c>
       <c r="G102" t="n">
-        <v>9419</v>
+        <v>23189</v>
       </c>
     </row>
     <row r="103">
@@ -22342,7 +22342,7 @@
         </is>
       </c>
       <c r="G129" t="n">
-        <v>28642</v>
+        <v>45007</v>
       </c>
     </row>
     <row r="130">

</xml_diff>

<commit_message>
Corregir precio CAÑERIAS AP 1/2" en Planta Antofagasta
Código 1002471 (Instalación Cañería Cu Alta Presión 1/2") tenía $9.382
en Antofagasta mientras los otros 4 centros (Copiapó, Arica, Iquique,
Calama) tienen $8.502 para el mismo código y diámetro — coincidía con
el precio de MP/BP a 1/2", parece un error de digitación cruzada entre
categorías. Se corrige a $8.502 para que quede uniforme en los 5 centros,
como el resto de las 79 combinaciones diámetro×centro en AP/MP/BP.
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAÑERIAS AP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAÑERIAS MP" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAÑERIAS BP" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERVICIO CAÑERIAS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONEXIONES" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OBRAS CIVILES" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NORMALIZACIONES" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUIPO COMPRA DIRECTA" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SERVICIO COMPRA DIRECTA" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="CAÑERIAS AP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CAÑERIAS MP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CAÑERIAS BP" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SERVICIO CAÑERIAS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CONEXIONES" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="OBRAS CIVILES" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="NORMALIZACIONES" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="EQUIPO COMPRA DIRECTA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SERVICIO COMPRA DIRECTA" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CAÑERIAS AP'!$A$1:$G$41</definedName>
@@ -1256,7 +1256,7 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>9382</v>
+        <v>8502</v>
       </c>
     </row>
     <row r="21" hidden="1">

</xml_diff>

<commit_message>
Corregir precio inconsistente en CAÑERIAS BP para códigos 1002478 y 1002527
Ambos códigos tenían $9.175 en la hoja CAÑERIAS BP (Arica, Iquique,
Antofagasta, Calama) pero $10.125 en CAÑERIAS MP para los mismos
centros y el mismo ítem. Se unifica a $10.125 en las 5 centros de
ambas hojas.
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -5725,7 +5725,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="4" hidden="1">
@@ -5765,7 +5765,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="5" hidden="1">
@@ -5805,7 +5805,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="6" hidden="1">
@@ -5845,7 +5845,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="7" hidden="1">
@@ -7485,7 +7485,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="48" hidden="1">
@@ -7525,7 +7525,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="49" hidden="1">
@@ -7565,7 +7565,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="50" hidden="1">
@@ -7605,7 +7605,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="51" hidden="1">
@@ -7645,7 +7645,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="52" hidden="1">

</xml_diff>

<commit_message>
Eliminar MANO OBRA INDUSTRIAL (1000690) de SERVICIO COMPRA DIRECTA
Traía un precio de $64.985.854 idéntico en los 5 centros, ~3.250 veces
el valor real ($20.000/hora) que usa ese mismo código en CONEXIONES,
NORMALIZACIONES, OBRAS CIVILES y SERVICIO CAÑERIAS. Claro error de
digitación/corrupción de datos.
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -31001,7 +31001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31289,12 +31289,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MANO OBRA INDUSTRIAL</t>
+          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>1000690</t>
+          <t>1001884</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -31318,18 +31318,18 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>64985854</v>
+        <v>8751547</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
+          <t>MONTAJE Y PUESTA EN MARCHA</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>1001884</t>
+          <t>1001949</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -31353,18 +31353,18 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>8751547</v>
+        <v>12086000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MONTAJE Y PUESTA EN MARCHA</t>
+          <t>REMOCION DE ESCOMBROS</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>1001949</t>
+          <t>1001431</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -31388,18 +31388,18 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>12086000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>REMOCION DE ESCOMBROS</t>
+          <t>SOPORTE TUBERIA DE 1" A 2"</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>1001431</t>
+          <t>1001229</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -31423,18 +31423,18 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>300000</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SOPORTE TUBERIA DE 1" A 2"</t>
+          <t>VIATICO TRASLADO</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>1001229</t>
+          <t>1000640</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -31458,18 +31458,18 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>550000</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>VIATICO TRASLADO</t>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>1000640</t>
+          <t>1001879</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -31493,18 +31493,18 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>450000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
+          <t>CELOSIA EN MURO CON TESTIGUERA</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>1001879</t>
+          <t>1000962</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -31519,27 +31519,27 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Oficina Ventas Arica</t>
+          <t>Oficina Ventas Calama</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0300</t>
+          <t>0600</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>250000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CELOSIA EN MURO CON TESTIGUERA</t>
+          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>1000962</t>
+          <t>1000038</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -31563,18 +31563,18 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>70000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
+          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>1000038</t>
+          <t>1000900</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -31598,18 +31598,18 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>110000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
+          <t>INSTALACION CELOSIA</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>1000900</t>
+          <t>1001861</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -31633,18 +31633,18 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>300000</v>
+        <v>4990</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>INSTALACION CELOSIA</t>
+          <t>INSTALACION DE LETREROS DE PELIGRO</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>1001861</t>
+          <t>1001923</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -31668,18 +31668,18 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>4990</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>INSTALACION DE LETREROS DE PELIGRO</t>
+          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>1001923</t>
+          <t>1000274</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -31703,18 +31703,18 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>80000</v>
+        <v>41206879</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
+          <t>MANO OBRA HABITACIONAL</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>1000274</t>
+          <t>1000770</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -31738,18 +31738,18 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>41206879</v>
+        <v>4050000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MANO OBRA HABITACIONAL</t>
+          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>1000770</t>
+          <t>1001884</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -31773,18 +31773,18 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>4050000</v>
+        <v>8751547</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MANO OBRA INDUSTRIAL</t>
+          <t>MONTAJE Y PUESTA EN MARCHA</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>1000690</t>
+          <t>1001949</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -31808,18 +31808,18 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>64985854</v>
+        <v>12086000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
+          <t>REMOCION DE ESCOMBROS</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>1001884</t>
+          <t>1001431</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -31843,18 +31843,18 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>8751547</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MONTAJE Y PUESTA EN MARCHA</t>
+          <t>SOPORTE TUBERIA DE 1" A 2"</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>1001949</t>
+          <t>1001229</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -31878,18 +31878,18 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>12086000</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>REMOCION DE ESCOMBROS</t>
+          <t>VIATICO TRASLADO</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>1001431</t>
+          <t>1000640</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -31913,18 +31913,18 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>300000</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SOPORTE TUBERIA DE 1" A 2"</t>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>1001229</t>
+          <t>1001879</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -31948,18 +31948,18 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>550000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>VIATICO TRASLADO</t>
+          <t>CELOSIA EN MURO CON TESTIGUERA</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>1000640</t>
+          <t>1000962</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -31974,27 +31974,27 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Oficina Ventas Copiapó</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>450000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
+          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>1001879</t>
+          <t>1000038</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -32009,27 +32009,27 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Oficina Ventas Copiapó</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>250000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CELOSIA EN MURO CON TESTIGUERA</t>
+          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>1000962</t>
+          <t>1000900</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -32053,18 +32053,18 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>70000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
+          <t>INSTALACION CELOSIA</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>1000038</t>
+          <t>1001861</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -32088,18 +32088,18 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>110000</v>
+        <v>4990</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
+          <t>INSTALACION DE LETREROS DE PELIGRO</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>1000900</t>
+          <t>1001923</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -32123,18 +32123,18 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>300000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>INSTALACION CELOSIA</t>
+          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>1001861</t>
+          <t>1000274</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -32158,18 +32158,18 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>4990</v>
+        <v>41206879</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>INSTALACION DE LETREROS DE PELIGRO</t>
+          <t>MANO OBRA HABITACIONAL</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>1001923</t>
+          <t>1000770</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -32193,18 +32193,18 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>80000</v>
+        <v>4050000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
+          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>1000274</t>
+          <t>1001884</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -32228,18 +32228,18 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>41206879</v>
+        <v>8751547</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MANO OBRA HABITACIONAL</t>
+          <t>MONTAJE Y PUESTA EN MARCHA</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>1000770</t>
+          <t>1001949</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -32263,18 +32263,18 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>4050000</v>
+        <v>12086000</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MANO OBRA INDUSTRIAL</t>
+          <t>REMOCION DE ESCOMBROS</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>1000690</t>
+          <t>1001431</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -32298,18 +32298,18 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>64985854</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
+          <t>SOPORTE TUBERIA DE 1" A 2"</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>1001884</t>
+          <t>1001229</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -32333,18 +32333,18 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>8751547</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MONTAJE Y PUESTA EN MARCHA</t>
+          <t>VIATICO TRASLADO</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>1001949</t>
+          <t>1000640</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -32368,18 +32368,18 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>12086000</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>REMOCION DE ESCOMBROS</t>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>1001431</t>
+          <t>1001879</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -32403,18 +32403,18 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>300000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SOPORTE TUBERIA DE 1" A 2"</t>
+          <t>CELOSIA EN MURO CON TESTIGUERA</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>1001229</t>
+          <t>1000962</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -32429,27 +32429,27 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>550000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>VIATICO TRASLADO</t>
+          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>1000640</t>
+          <t>1000038</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -32464,27 +32464,27 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>450000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
+          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>1001879</t>
+          <t>1000900</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -32499,27 +32499,27 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>250000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CELOSIA EN MURO CON TESTIGUERA</t>
+          <t>INSTALACION CELOSIA</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>1000962</t>
+          <t>1001861</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -32543,18 +32543,18 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>70000</v>
+        <v>4990</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
+          <t>INSTALACION DE LETREROS DE PELIGRO</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>1000038</t>
+          <t>1001923</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -32578,18 +32578,18 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>110000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
+          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>1000900</t>
+          <t>1000274</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -32613,18 +32613,18 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>300000</v>
+        <v>41206879</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>INSTALACION CELOSIA</t>
+          <t>MANO OBRA HABITACIONAL</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>1001861</t>
+          <t>1000770</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -32648,18 +32648,18 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>4990</v>
+        <v>4050000</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>INSTALACION DE LETREROS DE PELIGRO</t>
+          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>1001923</t>
+          <t>1001884</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -32683,18 +32683,18 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>80000</v>
+        <v>8751547</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
+          <t>MONTAJE Y PUESTA EN MARCHA</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>1000274</t>
+          <t>1001949</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -32718,18 +32718,18 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>41206879</v>
+        <v>12086000</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MANO OBRA HABITACIONAL</t>
+          <t>REMOCION DE ESCOMBROS</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>1000770</t>
+          <t>1001431</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -32753,18 +32753,18 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>4050000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MANO OBRA INDUSTRIAL</t>
+          <t>SOPORTE TUBERIA DE 1" A 2"</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>1000690</t>
+          <t>1001229</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -32788,18 +32788,18 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>64985854</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
+          <t>VIATICO TRASLADO</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>1001884</t>
+          <t>1000640</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -32823,18 +32823,18 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>8751547</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MONTAJE Y PUESTA EN MARCHA</t>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>1001949</t>
+          <t>1001879</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -32858,18 +32858,18 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>12086000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>REMOCION DE ESCOMBROS</t>
+          <t>CELOSIA EN MURO CON TESTIGUERA</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>1001431</t>
+          <t>1000962</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -32884,27 +32884,27 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Planta Antofagasta</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>0500</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G54" t="n">
-        <v>300000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SOPORTE TUBERIA DE 1" A 2"</t>
+          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
-          <t>1001229</t>
+          <t>1000038</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -32919,27 +32919,27 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Planta Antofagasta</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>0500</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G55" t="n">
-        <v>550000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>VIATICO TRASLADO</t>
+          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
-          <t>1000640</t>
+          <t>1000900</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -32954,27 +32954,27 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Planta Antofagasta</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>0500</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G56" t="n">
-        <v>450000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
+          <t>INSTALACION CELOSIA</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
-          <t>1001879</t>
+          <t>1001861</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -32989,27 +32989,27 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Planta Antofagasta</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>0500</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G57" t="n">
-        <v>250000</v>
+        <v>4990</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CELOSIA EN MURO CON TESTIGUERA</t>
+          <t>INSTALACION DE LETREROS DE PELIGRO</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
-          <t>1000962</t>
+          <t>1001923</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -33033,18 +33033,18 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>70000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
+          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>1000038</t>
+          <t>1000274</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -33068,18 +33068,18 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>110000</v>
+        <v>41206879</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
+          <t>MANO OBRA HABITACIONAL</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t>1000900</t>
+          <t>1000770</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -33103,18 +33103,18 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>300000</v>
+        <v>4050000</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>INSTALACION CELOSIA</t>
+          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>1001861</t>
+          <t>1001884</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -33138,18 +33138,18 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>4990</v>
+        <v>8751547</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>INSTALACION DE LETREROS DE PELIGRO</t>
+          <t>MONTAJE Y PUESTA EN MARCHA</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t>1001923</t>
+          <t>1001949</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -33173,18 +33173,18 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>80000</v>
+        <v>12086000</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
+          <t>REMOCION DE ESCOMBROS</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>1000274</t>
+          <t>1001431</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -33208,18 +33208,18 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>41206879</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MANO OBRA HABITACIONAL</t>
+          <t>SOPORTE TUBERIA DE 1" A 2"</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>1000770</t>
+          <t>1001229</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -33243,18 +33243,18 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>4050000</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MANO OBRA INDUSTRIAL</t>
+          <t>VIATICO TRASLADO</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>1000690</t>
+          <t>1000640</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -33278,18 +33278,18 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>64985854</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>1001884</t>
+          <t>1001879</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -33313,181 +33313,6 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>8751547</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>MONTAJE Y PUESTA EN MARCHA</t>
-        </is>
-      </c>
-      <c r="B67" s="1" t="inlineStr">
-        <is>
-          <t>1001949</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G67" t="n">
-        <v>12086000</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>REMOCION DE ESCOMBROS</t>
-        </is>
-      </c>
-      <c r="B68" s="1" t="inlineStr">
-        <is>
-          <t>1001431</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G68" t="n">
-        <v>300000</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>SOPORTE TUBERIA DE 1" A 2"</t>
-        </is>
-      </c>
-      <c r="B69" s="1" t="inlineStr">
-        <is>
-          <t>1001229</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G69" t="n">
-        <v>550000</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>VIATICO TRASLADO</t>
-        </is>
-      </c>
-      <c r="B70" s="1" t="inlineStr">
-        <is>
-          <t>1000640</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G70" t="n">
-        <v>450000</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
-        </is>
-      </c>
-      <c r="B71" s="1" t="inlineStr">
-        <is>
-          <t>1001879</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G71" t="n">
         <v>250000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Eliminar 5 ítems duplicados de SERVICIO COMPRA DIRECTA
Los códigos 1000640 (VIATICO TRASLADO), 1000900 (DECLARACION SALA DE
CALDERA SOBRE 70KW), 1001229 (SOPORTE TUBERIA DE 1" A 2"), 1001431
(REMOCION DE ESCOMBROS) e 1001923 (INSTALACION DE LETREROS DE PELIGRO)
ya existían en su hoja de categoría propia (Conexiones, Normalizaciones,
Servicio Cañerías, Obras Civiles) con precios distintos. Se eliminan
de Servicio Compra Directa para evitar ambigüedad de precio por código
duplicado entre categorías.
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -31001,7 +31001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31114,12 +31114,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
+          <t>INSTALACION CELOSIA</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>1000900</t>
+          <t>1001861</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -31143,18 +31143,18 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>300000</v>
+        <v>4990</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>INSTALACION CELOSIA</t>
+          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>1001861</t>
+          <t>1000274</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -31178,18 +31178,18 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>4990</v>
+        <v>41206879</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>INSTALACION DE LETREROS DE PELIGRO</t>
+          <t>MANO OBRA HABITACIONAL</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>1001923</t>
+          <t>1000770</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -31213,18 +31213,18 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>80000</v>
+        <v>4050000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
+          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>1000274</t>
+          <t>1001884</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -31248,18 +31248,18 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>41206879</v>
+        <v>8751547</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MANO OBRA HABITACIONAL</t>
+          <t>MONTAJE Y PUESTA EN MARCHA</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>1000770</t>
+          <t>1001949</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -31283,18 +31283,18 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>4050000</v>
+        <v>12086000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>1001884</t>
+          <t>1001879</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -31318,18 +31318,18 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>8751547</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MONTAJE Y PUESTA EN MARCHA</t>
+          <t>CELOSIA EN MURO CON TESTIGUERA</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>1001949</t>
+          <t>1000962</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -31344,27 +31344,27 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Oficina Ventas Arica</t>
+          <t>Oficina Ventas Calama</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0300</t>
+          <t>0600</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>12086000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>REMOCION DE ESCOMBROS</t>
+          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>1001431</t>
+          <t>1000038</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -31379,27 +31379,27 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Oficina Ventas Arica</t>
+          <t>Oficina Ventas Calama</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0300</t>
+          <t>0600</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>300000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SOPORTE TUBERIA DE 1" A 2"</t>
+          <t>INSTALACION CELOSIA</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>1001229</t>
+          <t>1001861</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -31414,27 +31414,27 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Oficina Ventas Arica</t>
+          <t>Oficina Ventas Calama</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0300</t>
+          <t>0600</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>550000</v>
+        <v>4990</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>VIATICO TRASLADO</t>
+          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>1000640</t>
+          <t>1000274</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -31449,27 +31449,27 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Oficina Ventas Arica</t>
+          <t>Oficina Ventas Calama</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0300</t>
+          <t>0600</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>450000</v>
+        <v>41206879</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
+          <t>MANO OBRA HABITACIONAL</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>1001879</t>
+          <t>1000770</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -31484,27 +31484,27 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Oficina Ventas Arica</t>
+          <t>Oficina Ventas Calama</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0300</t>
+          <t>0600</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>250000</v>
+        <v>4050000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CELOSIA EN MURO CON TESTIGUERA</t>
+          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>1000962</t>
+          <t>1001884</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -31528,18 +31528,18 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>70000</v>
+        <v>8751547</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
+          <t>MONTAJE Y PUESTA EN MARCHA</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>1000038</t>
+          <t>1001949</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -31563,18 +31563,18 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>110000</v>
+        <v>12086000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>1000900</t>
+          <t>1001879</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -31598,18 +31598,18 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>300000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>INSTALACION CELOSIA</t>
+          <t>CELOSIA EN MURO CON TESTIGUERA</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>1001861</t>
+          <t>1000962</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -31624,27 +31624,27 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Oficina Ventas Copiapó</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>4990</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>INSTALACION DE LETREROS DE PELIGRO</t>
+          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>1001923</t>
+          <t>1000038</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -31659,27 +31659,27 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Oficina Ventas Copiapó</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>80000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
+          <t>INSTALACION CELOSIA</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>1000274</t>
+          <t>1001861</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -31694,27 +31694,27 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Oficina Ventas Copiapó</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>41206879</v>
+        <v>4990</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MANO OBRA HABITACIONAL</t>
+          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>1000770</t>
+          <t>1000274</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -31729,27 +31729,27 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Oficina Ventas Copiapó</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>4050000</v>
+        <v>41206879</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
+          <t>MANO OBRA HABITACIONAL</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>1001884</t>
+          <t>1000770</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -31764,27 +31764,27 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Oficina Ventas Copiapó</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>8751547</v>
+        <v>4050000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MONTAJE Y PUESTA EN MARCHA</t>
+          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>1001949</t>
+          <t>1001884</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -31799,27 +31799,27 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Oficina Ventas Copiapó</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>12086000</v>
+        <v>8751547</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>REMOCION DE ESCOMBROS</t>
+          <t>MONTAJE Y PUESTA EN MARCHA</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>1001431</t>
+          <t>1001949</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -31834,27 +31834,27 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Oficina Ventas Copiapó</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>300000</v>
+        <v>12086000</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SOPORTE TUBERIA DE 1" A 2"</t>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>1001229</t>
+          <t>1001879</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -31869,27 +31869,27 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Oficina Ventas Copiapó</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0005</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>550000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VIATICO TRASLADO</t>
+          <t>CELOSIA EN MURO CON TESTIGUERA</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>1000640</t>
+          <t>1000962</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -31904,27 +31904,27 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>450000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
+          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>1001879</t>
+          <t>1000038</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -31939,27 +31939,27 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Oficina Ventas Calama</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0600</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>250000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CELOSIA EN MURO CON TESTIGUERA</t>
+          <t>INSTALACION CELOSIA</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>1000962</t>
+          <t>1001861</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -31974,27 +31974,27 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>70000</v>
+        <v>4990</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
+          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>1000038</t>
+          <t>1000274</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -32009,27 +32009,27 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>110000</v>
+        <v>41206879</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
+          <t>MANO OBRA HABITACIONAL</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>1000900</t>
+          <t>1000770</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -32044,27 +32044,27 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>300000</v>
+        <v>4050000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>INSTALACION CELOSIA</t>
+          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>1001861</t>
+          <t>1001884</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -32079,27 +32079,27 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>4990</v>
+        <v>8751547</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>INSTALACION DE LETREROS DE PELIGRO</t>
+          <t>MONTAJE Y PUESTA EN MARCHA</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>1001923</t>
+          <t>1001949</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -32114,27 +32114,27 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>80000</v>
+        <v>12086000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>1000274</t>
+          <t>1001879</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -32149,27 +32149,27 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Antofagasta</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0500</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>41206879</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MANO OBRA HABITACIONAL</t>
+          <t>CELOSIA EN MURO CON TESTIGUERA</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>1000770</t>
+          <t>1000962</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -32184,27 +32184,27 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>4050000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
+          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>1001884</t>
+          <t>1000038</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -32219,27 +32219,27 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>8751547</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MONTAJE Y PUESTA EN MARCHA</t>
+          <t>INSTALACION CELOSIA</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>1001949</t>
+          <t>1001861</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -32254,27 +32254,27 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>12086000</v>
+        <v>4990</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>REMOCION DE ESCOMBROS</t>
+          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>1001431</t>
+          <t>1000274</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -32289,27 +32289,27 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>300000</v>
+        <v>41206879</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SOPORTE TUBERIA DE 1" A 2"</t>
+          <t>MANO OBRA HABITACIONAL</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>1001229</t>
+          <t>1000770</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -32324,27 +32324,27 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>550000</v>
+        <v>4050000</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>VIATICO TRASLADO</t>
+          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>1000640</t>
+          <t>1001884</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -32359,27 +32359,27 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>450000</v>
+        <v>8751547</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
+          <t>MONTAJE Y PUESTA EN MARCHA</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>1001879</t>
+          <t>1001949</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -32394,27 +32394,27 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Oficina Ventas Copiapó</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>0005</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>250000</v>
+        <v>12086000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CELOSIA EN MURO CON TESTIGUERA</t>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>1000962</t>
+          <t>1001879</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -32429,890 +32429,15 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Planta Antofagasta</t>
+          <t>Planta Iquique</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>0500</t>
+          <t>0400</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>70000</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
-        </is>
-      </c>
-      <c r="B42" s="1" t="inlineStr">
-        <is>
-          <t>1000038</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>110000</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
-        </is>
-      </c>
-      <c r="B43" s="1" t="inlineStr">
-        <is>
-          <t>1000900</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>300000</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>INSTALACION CELOSIA</t>
-        </is>
-      </c>
-      <c r="B44" s="1" t="inlineStr">
-        <is>
-          <t>1001861</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>4990</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>INSTALACION DE LETREROS DE PELIGRO</t>
-        </is>
-      </c>
-      <c r="B45" s="1" t="inlineStr">
-        <is>
-          <t>1001923</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>80000</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
-        </is>
-      </c>
-      <c r="B46" s="1" t="inlineStr">
-        <is>
-          <t>1000274</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>41206879</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>MANO OBRA HABITACIONAL</t>
-        </is>
-      </c>
-      <c r="B47" s="1" t="inlineStr">
-        <is>
-          <t>1000770</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>4050000</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
-        </is>
-      </c>
-      <c r="B48" s="1" t="inlineStr">
-        <is>
-          <t>1001884</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>8751547</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>MONTAJE Y PUESTA EN MARCHA</t>
-        </is>
-      </c>
-      <c r="B49" s="1" t="inlineStr">
-        <is>
-          <t>1001949</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>12086000</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>REMOCION DE ESCOMBROS</t>
-        </is>
-      </c>
-      <c r="B50" s="1" t="inlineStr">
-        <is>
-          <t>1001431</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>300000</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>SOPORTE TUBERIA DE 1" A 2"</t>
-        </is>
-      </c>
-      <c r="B51" s="1" t="inlineStr">
-        <is>
-          <t>1001229</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>550000</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>VIATICO TRASLADO</t>
-        </is>
-      </c>
-      <c r="B52" s="1" t="inlineStr">
-        <is>
-          <t>1000640</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G52" t="n">
-        <v>450000</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
-        </is>
-      </c>
-      <c r="B53" s="1" t="inlineStr">
-        <is>
-          <t>1001879</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Planta Antofagasta</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>0500</t>
-        </is>
-      </c>
-      <c r="G53" t="n">
-        <v>250000</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>CELOSIA EN MURO CON TESTIGUERA</t>
-        </is>
-      </c>
-      <c r="B54" s="1" t="inlineStr">
-        <is>
-          <t>1000962</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G54" t="n">
-        <v>70000</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>CONEXION RED MATRIZ EXIST (POLIETILENO)</t>
-        </is>
-      </c>
-      <c r="B55" s="1" t="inlineStr">
-        <is>
-          <t>1000038</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G55" t="n">
-        <v>110000</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>DECLARACION SALA DE CALDERA SOBRE 70KW</t>
-        </is>
-      </c>
-      <c r="B56" s="1" t="inlineStr">
-        <is>
-          <t>1000900</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G56" t="n">
-        <v>300000</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>INSTALACION CELOSIA</t>
-        </is>
-      </c>
-      <c r="B57" s="1" t="inlineStr">
-        <is>
-          <t>1001861</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G57" t="n">
-        <v>4990</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>INSTALACION DE LETREROS DE PELIGRO</t>
-        </is>
-      </c>
-      <c r="B58" s="1" t="inlineStr">
-        <is>
-          <t>1001923</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G58" t="n">
-        <v>80000</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
-        </is>
-      </c>
-      <c r="B59" s="1" t="inlineStr">
-        <is>
-          <t>1000274</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G59" t="n">
-        <v>41206879</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>MANO OBRA HABITACIONAL</t>
-        </is>
-      </c>
-      <c r="B60" s="1" t="inlineStr">
-        <is>
-          <t>1000770</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G60" t="n">
-        <v>4050000</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>MONTAJE Y CONEXION NUEVA CALDERA</t>
-        </is>
-      </c>
-      <c r="B61" s="1" t="inlineStr">
-        <is>
-          <t>1001884</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G61" t="n">
-        <v>8751547</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>MONTAJE Y PUESTA EN MARCHA</t>
-        </is>
-      </c>
-      <c r="B62" s="1" t="inlineStr">
-        <is>
-          <t>1001949</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G62" t="n">
-        <v>12086000</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>REMOCION DE ESCOMBROS</t>
-        </is>
-      </c>
-      <c r="B63" s="1" t="inlineStr">
-        <is>
-          <t>1001431</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G63" t="n">
-        <v>300000</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>SOPORTE TUBERIA DE 1" A 2"</t>
-        </is>
-      </c>
-      <c r="B64" s="1" t="inlineStr">
-        <is>
-          <t>1001229</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G64" t="n">
-        <v>550000</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>VIATICO TRASLADO</t>
-        </is>
-      </c>
-      <c r="B65" s="1" t="inlineStr">
-        <is>
-          <t>1000640</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G65" t="n">
-        <v>450000</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
-        </is>
-      </c>
-      <c r="B66" s="1" t="inlineStr">
-        <is>
-          <t>1001879</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>SERVICIO COMPRA DIRECTA</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Planta Iquique</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>0400</t>
-        </is>
-      </c>
-      <c r="G66" t="n">
         <v>250000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar base_datos.xlsx con precios de cañería del DC 19512419 (Arica)
Se toma el DC como fuente de verdad para dos ítems de cañería en el
centro Arica: código 1002481 (Cu Media/Baja Presión 2", de $10.424 a
$11.503 en CAÑERIAS BP y MP) y código 1002474 (Cu Alta Presión 3/4",
de $8.502 a $9.382 en CAÑERIAS AP). Se revierte el proyecto de ejemplo
19512419 a esos mismos valores para quedar consistente con la base.

Con esto, la única diferencia restante entre el DC original y la Nota
de Venta es la corrección de material (pérdida no aplicada en 1 1/4"
y 2"), +$227.096.
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -1776,7 +1776,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="34" hidden="1">
@@ -4653,7 +4653,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>10424</v>
+        <v>11503</v>
       </c>
     </row>
     <row r="64" hidden="1">
@@ -8125,7 +8125,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>10424</v>
+        <v>11503</v>
       </c>
     </row>
     <row r="64" hidden="1">

</xml_diff>

<commit_message>
Unificar precios de cañería (2" MP/BP y AP 3/4") en todos los centros
Los ítems de las hojas CAÑERIAS AP/MP/BP tienen el mismo precio en
los 5 centros, así que se extiende a Copiapó, Iquique, Antofagasta y
Calama el valor ya confirmado con el DC 19512419 para Arica:
- 1002481 (Cu Media/Baja Presión 2"): $11.503
- 1002474 (Cu Alta Presión 3/4"): $9.382
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -1736,7 +1736,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="33" hidden="1">
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="35">
@@ -1856,7 +1856,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="36" hidden="1">
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="37" hidden="1">
@@ -4613,7 +4613,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>10424</v>
+        <v>11503</v>
       </c>
     </row>
     <row r="63" hidden="1">
@@ -4693,7 +4693,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>10424</v>
+        <v>11503</v>
       </c>
     </row>
     <row r="65" hidden="1">
@@ -4733,7 +4733,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>10424</v>
+        <v>11503</v>
       </c>
     </row>
     <row r="66" hidden="1">
@@ -4773,7 +4773,7 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>10424</v>
+        <v>11503</v>
       </c>
     </row>
     <row r="67" hidden="1">
@@ -8085,7 +8085,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>10424</v>
+        <v>11503</v>
       </c>
     </row>
     <row r="63" hidden="1">
@@ -8165,7 +8165,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>10424</v>
+        <v>11503</v>
       </c>
     </row>
     <row r="65" hidden="1">
@@ -8205,7 +8205,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>10424</v>
+        <v>11503</v>
       </c>
     </row>
     <row r="66" hidden="1">
@@ -8245,7 +8245,7 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>10424</v>
+        <v>11503</v>
       </c>
     </row>
     <row r="67" hidden="1">

</xml_diff>

<commit_message>
Agregar 19 ítems del DC 19512419 ausentes en base_datos.xlsx
Ítems industriales de Conexión (15), Obras Civiles (3) y
Normalización (1) que aparecían en el Detalle Comercial pero no
existían en ningún centro de la base. Se agregan con el mismo precio
en los 5 centros (Copiapó, Arica, Iquique, Antofagasta, Calama):

CONEXIONES: 1000184, 1000188, 1000088, 1000204, 1000255, 1000245,
1000243, 1000058, 1000262, 1001217, 1000244, 1000056, 1000965,
1001218, 1000154

OBRAS CIVILES: 1000611, 1001290, 1000022

NORMALIZACIONES: 1000820
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -9820,7 +9820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G149"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="12.5703125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -12416,6 +12416,2631 @@
       </c>
       <c r="G74" t="n">
         <v>20000</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEM INDUSTRIAL,RED EN 1 1/4"</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1000184</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>54955</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEM INDUSTRIAL,RED EN 1 1/4"</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1000184</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>54955</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEM INDUSTRIAL,RED EN 1 1/4"</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1000184</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>54955</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEM INDUSTRIAL,RED EN 1 1/4"</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1000184</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>54955</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEM INDUSTRIAL,RED EN 1 1/4"</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1000184</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>54955</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 2"</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1000188</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>85461</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 2"</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1000188</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>85461</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 2"</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1000188</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>85461</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 2"</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1000188</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>85461</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 2"</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1000188</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>85461</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>INTERCONEXION SERV. P/4 EST. AEREOS DE</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1000088</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>173373</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>INTERCONEXION SERV. P/4 EST. AEREOS DE</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1000088</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>173373</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>INTERCONEXION SERV. P/4 EST. AEREOS DE</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1000088</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>173373</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>INTERCONEXION SERV. P/4 EST. AEREOS DE</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1000088</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>173373</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>INTERCONEXION SERV. P/4 EST. AEREOS DE</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1000088</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>173373</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR PRIMERA ETAPA 1"</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1000204</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR PRIMERA ETAPA 1"</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1000204</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR PRIMERA ETAPA 1"</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1000204</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR PRIMERA ETAPA 1"</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1000204</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR PRIMERA ETAPA 1"</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1000204</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 3/4" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1000255</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 3/4" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1000255</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 3/4" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1000255</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 3/4" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1000255</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G98" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 3/4" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1000255</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G99" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1000245</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G100" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1000245</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G101" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1000245</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G102" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1000245</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G103" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1000245</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G104" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/4" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1000243</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G105" t="n">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/4" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1000243</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G106" t="n">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/4" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1000243</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G107" t="n">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/4" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1000243</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G108" t="n">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/4" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1000243</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G109" t="n">
+        <v>42000</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FLEXIBLES 3/4"</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1000058</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G110" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FLEXIBLES 3/4"</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1000058</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G111" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FLEXIBLES 3/4"</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1000058</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G112" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FLEXIBLES 3/4"</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1000058</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G113" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FLEXIBLES 3/4"</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1000058</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G114" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VAPORIZ 3/4" IN Y 1" OUT</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1000262</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G115" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VAPORIZ 3/4" IN Y 1" OUT</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1000262</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G116" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VAPORIZ 3/4" IN Y 1" OUT</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1000262</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G117" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VAPORIZ 3/4" IN Y 1" OUT</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1000262</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G118" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VAPORIZ 3/4" IN Y 1" OUT</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1000262</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G119" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>CONEXION FILTRO VAPORIZADOR H-1 1/4"</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1001217</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G120" t="n">
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>CONEXION FILTRO VAPORIZADOR H-1 1/4"</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1001217</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G121" t="n">
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>CONEXION FILTRO VAPORIZADOR H-1 1/4"</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1001217</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G122" t="n">
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>CONEXION FILTRO VAPORIZADOR H-1 1/4"</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1001217</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G123" t="n">
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>CONEXION FILTRO VAPORIZADOR H-1 1/4"</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1001217</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G124" t="n">
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/4" MED O BAJ PRE</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1000244</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G125" t="n">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/4" MED O BAJ PRE</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1000244</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G126" t="n">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/4" MED O BAJ PRE</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1000244</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G127" t="n">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/4" MED O BAJ PRE</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1000244</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G128" t="n">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/4" MED O BAJ PRE</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1000244</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G129" t="n">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FILTRO MEDIA PRESION 3/4"</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1000056</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G130" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FILTRO MEDIA PRESION 3/4"</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1000056</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G131" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FILTRO MEDIA PRESION 3/4"</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1000056</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G132" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FILTRO MEDIA PRESION 3/4"</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1000056</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G133" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FILTRO MEDIA PRESION 3/4"</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1000056</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G134" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>CONEXIÓN RED EXISTENTE 3/4" A 1"</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1000965</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G135" t="n">
+        <v>20213</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>CONEXIÓN RED EXISTENTE 3/4" A 1"</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1000965</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G136" t="n">
+        <v>20213</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>CONEXIÓN RED EXISTENTE 3/4" A 1"</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1000965</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G137" t="n">
+        <v>20213</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>CONEXIÓN RED EXISTENTE 3/4" A 1"</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1000965</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G138" t="n">
+        <v>20213</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>CONEXIÓN RED EXISTENTE 3/4" A 1"</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1000965</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G139" t="n">
+        <v>20213</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>CONEXION MANOMETRO ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1001218</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G140" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>CONEXION MANOMETRO ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1001218</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G141" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>CONEXION MANOMETRO ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1001218</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G142" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>CONEXION MANOMETRO ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1001218</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G143" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>CONEXION MANOMETRO ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1001218</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G144" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>CONEXIÓN MANOMETRO BAJA PRESI 0-60 MBAR</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1000154</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G145" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>CONEXIÓN MANOMETRO BAJA PRESI 0-60 MBAR</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1000154</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G146" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>CONEXIÓN MANOMETRO BAJA PRESI 0-60 MBAR</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1000154</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G147" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>CONEXIÓN MANOMETRO BAJA PRESI 0-60 MBAR</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1000154</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G148" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>CONEXIÓN MANOMETRO BAJA PRESI 0-60 MBAR</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1000154</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G149" t="n">
+        <v>7000</v>
       </c>
     </row>
   </sheetData>
@@ -12429,7 +15054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -14010,6 +16635,531 @@
       </c>
       <c r="G45" t="n">
         <v>3000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>METRO LINEAL DE REJA VERT. P/EST. AEREO</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1000611</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>METRO LINEAL DE REJA VERT. P/EST. AEREO</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1000611</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>METRO LINEAL DE REJA VERT. P/EST. AEREO</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1000611</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>METRO LINEAL DE REJA VERT. P/EST. AEREO</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1000611</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>METRO LINEAL DE REJA VERT. P/EST. AEREO</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1000611</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ARRIENDO-TRASL. EQUIPO HID. ALZA HOMBRE</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1001290</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ARRIENDO-TRASL. EQUIPO HID. ALZA HOMBRE</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1001290</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ARRIENDO-TRASL. EQUIPO HID. ALZA HOMBRE</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1001290</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ARRIENDO-TRASL. EQUIPO HID. ALZA HOMBRE</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1001290</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ARRIENDO-TRASL. EQUIPO HID. ALZA HOMBRE</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1001290</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>BASES Y ANCLAJE VAPORIZ-FILTRO DEC.H-10"</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1000022</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>BASES Y ANCLAJE VAPORIZ-FILTRO DEC.H-10"</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1000022</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BASES Y ANCLAJE VAPORIZ-FILTRO DEC.H-10"</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1000022</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>BASES Y ANCLAJE VAPORIZ-FILTRO DEC.H-10"</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>1000022</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>BASES Y ANCLAJE VAPORIZ-FILTRO DEC.H-10"</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1000022</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>70000</v>
       </c>
     </row>
   </sheetData>
@@ -14023,7 +17173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G108"/>
+  <dimension ref="A1:G113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="57.140625" customWidth="1" min="3" max="3"/>
@@ -17809,6 +20959,181 @@
       </c>
       <c r="G108" t="n">
         <v>65000</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>CERTIFICACION INTEGRAL INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1000820</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G109" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>CERTIFICACION INTEGRAL INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1000820</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G110" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>CERTIFICACION INTEGRAL INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1000820</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G111" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>CERTIFICACION INTEGRAL INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1000820</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G112" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>CERTIFICACION INTEGRAL INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1000820</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G113" t="n">
+        <v>150000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregar 10 códigos nuevos encontrados en 4 DC (Iquique, Copiapó, Antofagasta, Arica)
Ítems ausentes de la base, agregados con el mismo precio en los 5
centros a partir de los DC 19510789, 19519503, 19160327 y 19384780:

CONEXIONES: 1000206 (Regulador 2da etapa 1 1/2"), 1000630 (Regulador
etapa única), 1000073 (Horno de panadería), 1000964 (Cocina industrial
1"), 1000246 (Válv corte 1" media/baja), 1001219 (U. americana AP 3/4")

OBRAS CIVILES: 1000168 (Metro lineal excav/retape 1m), 1001206
(Zócalo cemento protección cañería), 1000219 (Reja estanque
superbalón 190)

SERVICIO CAÑERIAS: 1001227 (Protección planza cañería hasta 2")
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -9066,7 +9066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="22.42578125" customWidth="1" min="1" max="8"/>
@@ -10682,6 +10682,181 @@
       </c>
       <c r="G46" t="n">
         <v>1188</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PROTECCION PLANZA CAÑERIA HASTA 2"</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1001227</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PROTECCION PLANZA CAÑERIA HASTA 2"</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1001227</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PROTECCION PLANZA CAÑERIA HASTA 2"</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1001227</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>PROTECCION PLANZA CAÑERIA HASTA 2"</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1001227</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>PROTECCION PLANZA CAÑERIA HASTA 2"</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1001227</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>2150</v>
       </c>
     </row>
   </sheetData>
@@ -10695,7 +10870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G246"/>
+  <dimension ref="A1:G276"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="12.5703125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -19311,6 +19486,1056 @@
       </c>
       <c r="G246" t="n">
         <v>134565</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR SEGUNDA ETAPA 1 1/2"</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>1000206</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G247" t="n">
+        <v>55562</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR SEGUNDA ETAPA 1 1/2"</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>1000206</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G248" t="n">
+        <v>55562</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR SEGUNDA ETAPA 1 1/2"</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>1000206</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G249" t="n">
+        <v>55562</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR SEGUNDA ETAPA 1 1/2"</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>1000206</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G250" t="n">
+        <v>55562</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR SEGUNDA ETAPA 1 1/2"</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>1000206</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G251" t="n">
+        <v>55562</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR ETAPA UNICA</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>1000630</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G252" t="n">
+        <v>38500</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR ETAPA UNICA</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>1000630</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G253" t="n">
+        <v>38500</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR ETAPA UNICA</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>1000630</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G254" t="n">
+        <v>38500</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR ETAPA UNICA</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>1000630</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G255" t="n">
+        <v>38500</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR ETAPA UNICA</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>1000630</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G256" t="n">
+        <v>38500</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>CONEXIÓN HORNO DE PANADERIA</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>1000073</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G257" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>CONEXIÓN HORNO DE PANADERIA</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>1000073</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G258" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>CONEXIÓN HORNO DE PANADERIA</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>1000073</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G259" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>CONEXIÓN HORNO DE PANADERIA</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1000073</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>CONEXIÓN HORNO DE PANADERIA</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1000073</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G261" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>CONEXION COCINA INDUSTRIAL 1"</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>1000964</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G262" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>CONEXION COCINA INDUSTRIAL 1"</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>1000964</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G263" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>CONEXION COCINA INDUSTRIAL 1"</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>1000964</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G264" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>CONEXION COCINA INDUSTRIAL 1"</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>1000964</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G265" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>CONEXION COCINA INDUSTRIAL 1"</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>1000964</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G266" t="n">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1" MEDIA O BAJA PRES</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>1000246</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G267" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1" MEDIA O BAJA PRES</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>1000246</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G268" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1" MEDIA O BAJA PRES</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>1000246</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G269" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1" MEDIA O BAJA PRES</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>1000246</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G270" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1" MEDIA O BAJA PRES</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1000246</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G271" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>CONEXION U.AMERICANA AP HASTA 3/4"</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>1001219</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G272" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>CONEXION U.AMERICANA AP HASTA 3/4"</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>1001219</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G273" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>CONEXION U.AMERICANA AP HASTA 3/4"</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>1001219</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G274" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>CONEXION U.AMERICANA AP HASTA 3/4"</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>1001219</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G275" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>CONEXION U.AMERICANA AP HASTA 3/4"</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>1001219</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G276" t="n">
+        <v>38000</v>
       </c>
     </row>
   </sheetData>
@@ -19324,7 +20549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:G131"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -23390,6 +24615,531 @@
       </c>
       <c r="G116" t="n">
         <v>120000</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>METRO LINEAL EXCAV,PROTECC Y RETAPE 1M</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1000168</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G117" t="n">
+        <v>5559</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>METRO LINEAL EXCAV,PROTECC Y RETAPE 1M</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1000168</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G118" t="n">
+        <v>5559</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>METRO LINEAL EXCAV,PROTECC Y RETAPE 1M</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1000168</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G119" t="n">
+        <v>5559</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>METRO LINEAL EXCAV,PROTECC Y RETAPE 1M</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1000168</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G120" t="n">
+        <v>5559</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>METRO LINEAL EXCAV,PROTECC Y RETAPE 1M</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1000168</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G121" t="n">
+        <v>5559</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>ZOCALO CEMENTO PROTECCION CAÑERIA</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1001206</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G122" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>ZOCALO CEMENTO PROTECCION CAÑERIA</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1001206</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G123" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>ZOCALO CEMENTO PROTECCION CAÑERIA</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1001206</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G124" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>ZOCALO CEMENTO PROTECCION CAÑERIA</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1001206</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G125" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>ZOCALO CEMENTO PROTECCION CAÑERIA</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1001206</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G126" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>REJA ESTANQUE SUPERBALON 190</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1000219</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G127" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>REJA ESTANQUE SUPERBALON 190</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1000219</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G128" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>REJA ESTANQUE SUPERBALON 190</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1000219</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G129" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>REJA ESTANQUE SUPERBALON 190</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1000219</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G130" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>REJA ESTANQUE SUPERBALON 190</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1000219</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G131" t="n">
+        <v>200000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corregir precio placeholder de INSTALACION DE LETREROS DE PELIGRO (1001923)
Quedaba en \$1 en los 5 centros de OBRAS CIVILES (arrastrado desde el
relleno por moda anterior, que propagó un valor erróneo). Se actualiza
a \$200.000 según el DC 19512419 (Arica), confirmado como el valor
vigente frente a otro DC más antiguo que traía \$60.000.

1000046 (Detección Escape) se deja sin cambios en \$15.000: el DC
19519503 (Copiapó) que traía \$7.500 se determinó que era el error,
no la base.
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -21114,7 +21114,7 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="17">
@@ -21674,7 +21674,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="33">
@@ -23809,7 +23809,7 @@
         </is>
       </c>
       <c r="G93" t="n">
-        <v>1</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="94">
@@ -23844,7 +23844,7 @@
         </is>
       </c>
       <c r="G94" t="n">
-        <v>1</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="95">
@@ -23879,7 +23879,7 @@
         </is>
       </c>
       <c r="G95" t="n">
-        <v>1</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="96">

</xml_diff>

<commit_message>
Agregar cañería de acero LAP10AC (1", 3/4", 1 1/4") a CAÑERIAS AP
Mismo precio en los 5 centros: el precio de instalación ya incluye el
material, por eso va a precio fijo igual que la cañería de cobre y no
debe sumarse material Impovar (ya excluido en obtenerMaterialCañeria()).
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="37.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2097,6 +2097,606 @@
       </c>
       <c r="H41" t="n">
         <v>8502</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LAP10AC 1" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1000099</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>16145</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>LAP10AC 1" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1000099</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>16145</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>LAP10AC 1" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1000099</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>16145</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>LAP10AC 1" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1000099</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>16145</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>LAP10AC 1" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1000099</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>16145</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LAP10AC 3/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1000104</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>13173</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>LAP10AC 3/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1000104</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>13173</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>LAP10AC 3/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1000104</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>13173</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>LAP10AC 3/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1000104</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>13173</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>LAP10AC 3/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1000104</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>13173</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>LAP10AC 1 1/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1000098</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>18826</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>LAP10AC 1 1/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1000098</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>18826</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>LAP10AC 1 1/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1000098</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>18826</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>LAP10AC 1 1/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1000098</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>18826</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>LAP10AC 1 1/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1000098</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>18826</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregar códigos 1000186 y 1000181 del DC 19339040 a base_datos.xlsx
El DC 19339040 (Panificadora Heriberto Samit, Alto Hospicio - Planta
Iquique) trae dos códigos que no existían en ningún centro:
- 1000186 CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 1/2" (CONEXIONES, $55.000)
- 1000181 PROTECCION METALICA PARA REGULADOR (OBRAS CIVILES, $40.000)

Se agregan a los 5 centros con precio unificado, siguiendo la cobertura
completa existente. El resto de los 21 ítems SOLPED del DC ya estaba en
la base con los mismos precios (23/23 cuadran para Planta Iquique).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CpsrjGmbDGRie5TVH4b2fw
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -11470,7 +11470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G276"/>
+  <dimension ref="A1:G281"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="12.5703125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -21136,6 +21136,181 @@
       </c>
       <c r="G276" t="n">
         <v>38000</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 1/2"</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>1000186</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G277" t="n">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 1/2"</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>1000186</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G278" t="n">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 1/2"</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>1000186</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G279" t="n">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 1/2"</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>1000186</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G280" t="n">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 1/2"</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>1000186</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G281" t="n">
+        <v>55000</v>
       </c>
     </row>
   </sheetData>
@@ -21149,7 +21324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G131"/>
+  <dimension ref="A1:G136"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -25740,6 +25915,181 @@
       </c>
       <c r="G131" t="n">
         <v>200000</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>PROTECCION METALICA PARA REGULADOR</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="G132" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>PROTECCION METALICA PARA REGULADOR</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="G133" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>PROTECCION METALICA PARA REGULADOR</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="G134" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>PROTECCION METALICA PARA REGULADOR</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="G135" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>PROTECCION METALICA PARA REGULADOR</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G136" t="n">
+        <v>40000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>